<commit_message>
消融表换用新 w/o CDIS 臂 REMO_NoCDIS_REMOSelection
- 把 §4.3 消融表的 w/o CDIS 列数据源由 REMO_noBatchDict_noCDIS 换成本次新跑的
  REMO_NoCDIS_REMOSelection（16 题 × M=10/20 × 20 跑、N=100、请求 D=30（WFG2/3 实际 31）、
  maxFE=300、save=30；种子 20260912 + M*1e5 + 1000*题号 + run，与前一臂同一套）。
- experiments/ablation/sources/ 两份工作簿替换为新版；build_remo_reference.py 的表注
  改按新臂机制描述；table_ablation_igdp.tex 相应重新生成。
- 计数（相对 REMO）：w/o CDIS 由 19/2/11 变为 18/1/13；Full 28/2/2 与 w/o PAQC 20/1/11
  不变。两个未换臂逐格复现原数字，作为管线自校验。
- HPDC-MaOEA.tex §4.3：改写 w/o CDIS 控制的机制描述（保留 PAQC，整个 CDIS 换成本地 REMO
  原版候选模块，两个准则与模式切换均不存在），并把 DTLZ6/DTLZ7 的均值结论同步为
  两个目标数都低于 Full。
- 新增算法 REMO_NoCDIS_REMOSelection 及其 runner / 出表 / 校验脚本；experiments/ggp 下
  两份历史记录补充 2026-10-09 更正说明，不改写原记录。
- 验证：build_remo_reference.py --check 通过；pdflatex 两遍无错误、无未定义引用，
  仍为 16 页（与改动前 HEAD 编译结果一致）。
</commit_message>
<xml_diff>
--- a/论文写作/experiments/ablation/sources/nobatchdict以RMEO为基准二十目标IGDp.xlsx
+++ b/论文写作/experiments/ablation/sources/nobatchdict以RMEO为基准二十目标IGDp.xlsx
@@ -525,7 +525,7 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>7.6982e+1 (1.67e+1) +</t>
+          <t>7.9996e+1 (1.78e+1) +</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>9.1620e-1 (7.12e-2) =</t>
+          <t>9.0679e-1 (7.10e-2) =</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>3.4770e+2 (5.32e+1) =</t>
+          <t>3.1636e+2 (6.19e+1) +</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
@@ -635,14 +635,14 @@
       <c r="E5" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>7.1116e-1 (6.37e-2) +</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>7.1116e-1 (5.17e-2) +</t>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>7.4363e-1 (5.85e-2) =</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2.5455e-1 (7.92e-2) +</t>
+          <t>2.6929e-1 (7.47e-2) +</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>6.1597e+0 (9.18e-1) +</t>
+          <t>6.2089e+0 (6.57e-1) +</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
@@ -752,14 +752,14 @@
       <c r="E8" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>2.2885e+1 (4.26e+0) +</t>
         </is>
       </c>
-      <c r="G8" s="1" t="inlineStr">
-        <is>
-          <t>2.3639e+1 (7.57e+0) +</t>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2.1692e+1 (6.68e+0) +</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>4.1445e+0 (1.20e-1) +</t>
+          <t>4.1669e+0 (1.03e-1) +</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>4.7975e+0 (1.25e+0) +</t>
+          <t>3.9062e+0 (6.18e-1) +</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>2.4942e+0 (1.35e-1) -</t>
+          <t>2.4252e+0 (1.43e-1) -</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>2.2100e+1 (1.33e+0) =</t>
+          <t>2.2246e+1 (1.16e+0) =</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>2.1112e+1 (1.22e+0) =</t>
+          <t>2.0716e+1 (1.25e+0) =</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>1.6793e+1 (1.14e+0) +</t>
+          <t>1.7174e+1 (8.30e-1) +</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
-          <t>1.8214e+1 (1.03e+0) +</t>
+          <t>1.8237e+1 (1.04e+0) +</t>
         </is>
       </c>
       <c r="H15" s="1" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>1.8102e+1 (7.66e-1) +</t>
+          <t>1.8869e+1 (6.65e-1) +</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
-          <t>2.2623e+1 (1.06e+0) =</t>
+          <t>2.2417e+1 (1.22e+0) =</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">

</xml_diff>